<commit_message>
allAnswers_df stores answers. Bug fixed re points vector.
</commit_message>
<xml_diff>
--- a/Allsmall.xlsx
+++ b/Allsmall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\Machinegrading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CF01DAF-A143-4F47-AAC5-AFE8F8B2EBC7}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="32" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3E73B2-AED2-4719-BAC3-48DEB4792DCD}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="32" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11856" windowHeight="5676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,52 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>TRAN KHANH N</t>
+  </si>
+  <si>
+    <t>10310004130104202442213422</t>
+  </si>
+  <si>
+    <t>vC: 14, 16</t>
+  </si>
+  <si>
+    <t>10310034130102212442213422</t>
+  </si>
+  <si>
+    <t>vC: 7</t>
+  </si>
+  <si>
+    <t>HAO SHIRA</t>
+  </si>
+  <si>
+    <t>RUTAYISIRE DIANDRY A</t>
+  </si>
+  <si>
+    <t>10303032430441314203221120</t>
+  </si>
+  <si>
+    <t>vA: 7, 13, 19, 23</t>
+  </si>
+  <si>
+    <t>RUIZ TYLER J</t>
+  </si>
+  <si>
+    <t>10303022410421214211220120</t>
+  </si>
+  <si>
+    <t>vA: 10, 15, 20, 23</t>
+  </si>
+  <si>
+    <t>JIANG JASMINE</t>
+  </si>
+  <si>
+    <t>10303022430421314203223120</t>
+  </si>
+  <si>
+    <t>vA: 19</t>
+  </si>
   <si>
     <t>SHIELDS TIFFANY</t>
   </si>
@@ -56,88 +101,13 @@
     <t>vA: 1, 4, 8</t>
   </si>
   <si>
-    <t>TRAN KHANH N</t>
-  </si>
-  <si>
-    <t>10310004130104202442213422</t>
-  </si>
-  <si>
-    <t>vC: 14, 16</t>
-  </si>
-  <si>
-    <t>10310034130102212442213422</t>
-  </si>
-  <si>
-    <t>vC: 7</t>
-  </si>
-  <si>
-    <t>GIORDANO SOPHIA</t>
+    <t>SHIN DANIEL</t>
+  </si>
+  <si>
+    <t>10410034131102212442210422</t>
   </si>
   <si>
     <t>vC: 3, 7, 11, 23</t>
-  </si>
-  <si>
-    <t>SHIN DANIEL</t>
-  </si>
-  <si>
-    <t>10410034131102212442210422</t>
-  </si>
-  <si>
-    <t>HAO SHIRA</t>
-  </si>
-  <si>
-    <t>ROCHA TRISTA N</t>
-  </si>
-  <si>
-    <t>21014123334112030121420101</t>
-  </si>
-  <si>
-    <t>vB: 5, 6, 9, 11</t>
-  </si>
-  <si>
-    <t>DAVIS ALEAH N</t>
-  </si>
-  <si>
-    <t>21013103230113031121430101</t>
-  </si>
-  <si>
-    <t>vB: 6, 7, 9, 14, 17, 22</t>
-  </si>
-  <si>
-    <t>SMITH</t>
-  </si>
-  <si>
-    <t>10331022430421314213223100</t>
-  </si>
-  <si>
-    <t>vA: 4, 5, 25</t>
-  </si>
-  <si>
-    <t>RUIZ TYLER J</t>
-  </si>
-  <si>
-    <t>10303022410421214211220120</t>
-  </si>
-  <si>
-    <t>vA: 10, 15, 20, 23</t>
-  </si>
-  <si>
-    <t>RUTAYISIRE DIANDRY A</t>
-  </si>
-  <si>
-    <t>10303032430441314203221120</t>
-  </si>
-  <si>
-    <t>vA: 7, 13, 19, 23</t>
-  </si>
-  <si>
-    <t>JIANG JASMINE</t>
-  </si>
-  <si>
-    <t>10303022430421314203223120</t>
-  </si>
-  <si>
-    <t>vA: 19</t>
   </si>
 </sst>
 </file>
@@ -180,7 +150,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -522,13 +502,13 @@
         <v>1001</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E1">
         <v>24</v>
@@ -543,7 +523,7 @@
       </c>
       <c r="J1">
         <f>100*AVERAGE(H:H)/72</f>
-        <v>95.833333333333329</v>
+        <v>97.023809523809533</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -551,23 +531,23 @@
         <v>1002</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>25</v>
       </c>
       <c r="F2">
-        <f t="shared" ref="F2:F65" si="0">E2*3</f>
+        <f t="shared" ref="F2:F7" si="0">E2*3</f>
         <v>75</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H65" si="1">F2-G2</f>
+        <f t="shared" ref="H2:H7" si="1">F2-G2</f>
         <v>75</v>
       </c>
     </row>
@@ -576,13 +556,13 @@
         <v>1003</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E3">
         <v>22</v>
@@ -601,13 +581,13 @@
         <v>1004</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>22</v>
@@ -626,13 +606,13 @@
         <v>1005</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>25</v>
@@ -651,13 +631,13 @@
         <v>1006</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E6">
         <v>23</v>
@@ -676,13 +656,13 @@
         <v>1007</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E7">
         <v>22</v>
@@ -697,104 +677,24 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>1008</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8">
-        <v>20</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="H8">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>1009</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9">
-        <v>23</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>69</v>
-      </c>
-      <c r="H9">
-        <f t="shared" si="1"/>
-        <v>69</v>
-      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>1010</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10">
-        <v>22</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-      <c r="H10">
-        <f t="shared" si="1"/>
-        <v>66</v>
-      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>1012</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11">
-        <v>25</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="H11">
-        <f t="shared" si="1"/>
-        <v>75</v>
-      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
@@ -2070,7 +1970,10 @@
   <sortState ref="A1:E265">
     <sortCondition ref="A1:A265"/>
   </sortState>
-  <conditionalFormatting sqref="A1:A1048576">
+  <conditionalFormatting sqref="A8:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A7">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
analyse_items added which can analyse no of correct answers etc separately for each version. fixed bug that caused QIDs[0] to be incremented
</commit_message>
<xml_diff>
--- a/Allsmall.xlsx
+++ b/Allsmall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souri\Dropbox\Machinegrading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3E73B2-AED2-4719-BAC3-48DEB4792DCD}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="32" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2E5D0A-C8B2-49CF-8E95-43A9800F2012}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="32" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11856" windowHeight="5676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>TRAN KHANH N</t>
   </si>
@@ -81,33 +81,6 @@
   </si>
   <si>
     <t>vA: 10, 15, 20, 23</t>
-  </si>
-  <si>
-    <t>JIANG JASMINE</t>
-  </si>
-  <si>
-    <t>10303022430421314203223120</t>
-  </si>
-  <si>
-    <t>vA: 19</t>
-  </si>
-  <si>
-    <t>SHIELDS TIFFANY</t>
-  </si>
-  <si>
-    <t>20333021430421314213223120</t>
-  </si>
-  <si>
-    <t>vA: 1, 4, 8</t>
-  </si>
-  <si>
-    <t>SHIN DANIEL</t>
-  </si>
-  <si>
-    <t>10410034131102212442210422</t>
-  </si>
-  <si>
-    <t>vC: 3, 7, 11, 23</t>
   </si>
 </sst>
 </file>
@@ -523,7 +496,7 @@
       </c>
       <c r="J1">
         <f>100*AVERAGE(H:H)/72</f>
-        <v>97.023809523809533</v>
+        <v>96.875</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -602,79 +575,19 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>1005</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5">
-        <v>25</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="H5">
-        <f t="shared" si="1"/>
-        <v>75</v>
-      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>1006</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6">
-        <v>23</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="0"/>
-        <v>69</v>
-      </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
-        <v>69</v>
-      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>1007</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7">
-        <v>22</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-      <c r="H7">
-        <f t="shared" si="1"/>
-        <v>66</v>
-      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>

</xml_diff>